<commit_message>
Millora del network i dades a excel 'edges'
</commit_message>
<xml_diff>
--- a/data/network/nodes.xlsx
+++ b/data/network/nodes.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ArnauCoronado\Documents_local\euromed\sxs\data\network\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D2C78DD4-70B3-488D-91B7-71FE5419075F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{71B7DB7E-5C4B-4DD6-9853-73DED48DA7CF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{306F75E9-4DFE-4518-8798-1CA0D2BB102C}"/>
   </bookViews>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="172" uniqueCount="13">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="220" uniqueCount="58">
   <si>
     <t>source</t>
   </si>
@@ -63,9 +63,6 @@
     <t>bomba</t>
   </si>
   <si>
-    <t>intercanviador</t>
-  </si>
-  <si>
     <t>ramificació</t>
   </si>
   <si>
@@ -79,16 +76,160 @@
   </si>
   <si>
     <t>chiller</t>
+  </si>
+  <si>
+    <t>colector</t>
+  </si>
+  <si>
+    <t>1</t>
+  </si>
+  <si>
+    <t>Y-120</t>
+  </si>
+  <si>
+    <t>Y-160</t>
+  </si>
+  <si>
+    <t>Y-170</t>
+  </si>
+  <si>
+    <t>Y-180 (a)</t>
+  </si>
+  <si>
+    <t>Y-180 (b)</t>
+  </si>
+  <si>
+    <t>Y-190 (a)</t>
+  </si>
+  <si>
+    <t>Y-190 (b)</t>
+  </si>
+  <si>
+    <t>EI-101</t>
+  </si>
+  <si>
+    <t>EI-102</t>
+  </si>
+  <si>
+    <t>EI-150</t>
+  </si>
+  <si>
+    <t>EI-801</t>
+  </si>
+  <si>
+    <t>EI-806</t>
+  </si>
+  <si>
+    <t>EI-901</t>
+  </si>
+  <si>
+    <t>EI-906</t>
+  </si>
+  <si>
+    <t>PI-303</t>
+  </si>
+  <si>
+    <t>PI-304</t>
+  </si>
+  <si>
+    <t>PI-601</t>
+  </si>
+  <si>
+    <t>LI-651</t>
+  </si>
+  <si>
+    <t>LI-671</t>
+  </si>
+  <si>
+    <t>VI-710</t>
+  </si>
+  <si>
+    <t>VI-740</t>
+  </si>
+  <si>
+    <t>VI-810</t>
+  </si>
+  <si>
+    <t>SS-600</t>
+  </si>
+  <si>
+    <t>EI-701</t>
+  </si>
+  <si>
+    <t>SS-801</t>
+  </si>
+  <si>
+    <t>SS-802</t>
+  </si>
+  <si>
+    <t>BV-104</t>
+  </si>
+  <si>
+    <t>BV-105</t>
+  </si>
+  <si>
+    <t>BV-106</t>
+  </si>
+  <si>
+    <t>BV-107</t>
+  </si>
+  <si>
+    <t>BV-108</t>
+  </si>
+  <si>
+    <t>BV-109</t>
+  </si>
+  <si>
+    <t>EI-1001</t>
+  </si>
+  <si>
+    <t>EI-1006</t>
+  </si>
+  <si>
+    <t>SS-1000</t>
+  </si>
+  <si>
+    <t>SS-3000</t>
+  </si>
+  <si>
+    <t>SI-2107</t>
+  </si>
+  <si>
+    <t>SI-2207</t>
+  </si>
+  <si>
+    <t>PK-201</t>
+  </si>
+  <si>
+    <t>PK-202A</t>
+  </si>
+  <si>
+    <t>SI-6002</t>
+  </si>
+  <si>
+    <t>intercambiador</t>
+  </si>
+  <si>
+    <t>4600.02</t>
+  </si>
+  <si>
+    <t>4600.01</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="1" x14ac:knownFonts="1">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="8"/>
       <name val="Aptos Narrow"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -451,1236 +592,1568 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9701035B-20B7-437C-B875-CAFA64730628}">
-  <dimension ref="A1:E87"/>
+  <dimension ref="A1:F89"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="10" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="13.6640625" customWidth="1"/>
+    <col min="2" max="2" width="10" customWidth="1"/>
+    <col min="3" max="3" width="13.6640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>1</v>
       </c>
       <c r="B1" t="s">
+        <v>4</v>
+      </c>
+      <c r="C1" t="s">
         <v>5</v>
       </c>
-      <c r="C1" t="s">
+      <c r="D1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" t="s">
+      <c r="E1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" t="s">
+      <c r="F1" t="s">
         <v>4</v>
       </c>
     </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A2" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="B2" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="C2">
+        <v>9</v>
+      </c>
+      <c r="B2" t="s">
+        <v>12</v>
+      </c>
+      <c r="C2" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="D2">
         <v>0.22600000000000001</v>
       </c>
-      <c r="D2">
+      <c r="E2">
         <v>5.5123999999999999E-2</v>
       </c>
     </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A3" s="1">
+    <row r="3" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A3" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="B3" s="1" t="str">
+        <f>A3</f>
         <v>1</v>
       </c>
-      <c r="B3" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="C3">
+      <c r="C3" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="D3">
         <v>0.221</v>
       </c>
-      <c r="D3">
+      <c r="E3">
         <v>0.14346300000000001</v>
       </c>
     </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A4" s="1">
         <v>2</v>
       </c>
-      <c r="B4" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="C4">
+      <c r="B4" s="1">
+        <f t="shared" ref="B4:B26" si="0">A4</f>
+        <v>2</v>
+      </c>
+      <c r="C4" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="D4">
         <v>0.25800000000000001</v>
       </c>
-      <c r="D4">
+      <c r="E4">
         <v>0.14982300000000001</v>
       </c>
     </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A5" s="1">
         <v>3</v>
       </c>
-      <c r="B5" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="C5">
+      <c r="B5" s="1">
+        <f t="shared" si="0"/>
+        <v>3</v>
+      </c>
+      <c r="C5" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="D5">
         <v>0.28499999999999998</v>
       </c>
-      <c r="D5">
+      <c r="E5">
         <v>0.15335699999999999</v>
       </c>
     </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A6" s="1">
         <v>4</v>
       </c>
-      <c r="B6" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="C6">
+      <c r="B6" s="1">
+        <f t="shared" si="0"/>
+        <v>4</v>
+      </c>
+      <c r="C6" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="D6">
         <v>0.33700000000000002</v>
       </c>
-      <c r="D6">
+      <c r="E6">
         <v>0.16183700000000001</v>
       </c>
     </row>
-    <row r="7" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A7" s="1">
         <v>5</v>
       </c>
-      <c r="B7" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="C7">
+      <c r="B7" s="1">
+        <f t="shared" si="0"/>
+        <v>5</v>
+      </c>
+      <c r="C7" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="D7">
         <v>0.42399999999999999</v>
       </c>
-      <c r="D7">
+      <c r="E7">
         <v>0.176678</v>
       </c>
     </row>
-    <row r="8" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A8" s="1">
         <v>6</v>
       </c>
-      <c r="B8" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="C8">
+      <c r="B8" s="1">
+        <f t="shared" si="0"/>
+        <v>6</v>
+      </c>
+      <c r="C8" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="D8">
         <v>0.44500000000000001</v>
       </c>
-      <c r="D8">
+      <c r="E8">
         <v>0.37597199999999997</v>
       </c>
     </row>
-    <row r="9" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A9" s="1">
         <v>7</v>
       </c>
-      <c r="B9" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="C9">
+      <c r="B9" s="1">
+        <f t="shared" si="0"/>
+        <v>7</v>
+      </c>
+      <c r="C9" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="D9">
         <v>0.44600000000000001</v>
       </c>
-      <c r="D9">
+      <c r="E9">
         <v>0.39505299999999999</v>
       </c>
     </row>
-    <row r="10" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A10" s="1">
         <v>8</v>
       </c>
-      <c r="B10" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="C10">
+      <c r="B10" s="1">
+        <f t="shared" si="0"/>
+        <v>8</v>
+      </c>
+      <c r="C10" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="D10">
         <v>0.44350000000000001</v>
       </c>
-      <c r="D10">
+      <c r="E10">
         <v>0.41978799999999999</v>
       </c>
     </row>
-    <row r="11" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A11" s="1">
         <v>9</v>
       </c>
-      <c r="B11" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="C11">
+      <c r="B11" s="1">
+        <f t="shared" si="0"/>
+        <v>9</v>
+      </c>
+      <c r="C11" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="D11">
         <v>0.442</v>
       </c>
-      <c r="D11">
+      <c r="E11">
         <v>0.44523000000000001</v>
       </c>
     </row>
-    <row r="12" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A12" s="1">
         <v>10</v>
       </c>
-      <c r="B12" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="C12">
+      <c r="B12" s="1">
+        <f t="shared" si="0"/>
+        <v>10</v>
+      </c>
+      <c r="C12" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="D12">
         <v>0.4395</v>
       </c>
-      <c r="D12">
+      <c r="E12">
         <v>0.47915200000000002</v>
       </c>
     </row>
-    <row r="13" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A13" s="1">
         <v>11</v>
       </c>
-      <c r="B13" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="C13">
+      <c r="B13" s="1">
+        <f t="shared" si="0"/>
+        <v>11</v>
+      </c>
+      <c r="C13" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="D13">
         <v>0.439</v>
       </c>
-      <c r="D13">
+      <c r="E13">
         <v>0.49823299999999998</v>
       </c>
     </row>
-    <row r="14" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A14" s="1">
         <v>12</v>
       </c>
-      <c r="B14" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="C14">
+      <c r="B14" s="1">
+        <f t="shared" si="0"/>
+        <v>12</v>
+      </c>
+      <c r="C14" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="D14">
         <v>0.42349999999999999</v>
       </c>
-      <c r="D14">
+      <c r="E14">
         <v>0.497527</v>
       </c>
     </row>
-    <row r="15" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A15" s="1">
         <v>13</v>
       </c>
-      <c r="B15" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="C15">
+      <c r="B15" s="1">
+        <f t="shared" si="0"/>
+        <v>13</v>
+      </c>
+      <c r="C15" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="D15">
         <v>0.39700000000000002</v>
       </c>
-      <c r="D15">
+      <c r="E15">
         <v>0.49611300000000003</v>
       </c>
     </row>
-    <row r="16" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A16" s="1">
         <v>14</v>
       </c>
-      <c r="B16" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="C16">
+      <c r="B16" s="1">
+        <f t="shared" si="0"/>
+        <v>14</v>
+      </c>
+      <c r="C16" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="D16">
         <v>0.3765</v>
       </c>
-      <c r="D16">
+      <c r="E16">
         <v>0.56749099999999997</v>
       </c>
     </row>
-    <row r="17" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A17" s="1">
         <v>15</v>
       </c>
-      <c r="B17" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="C17">
+      <c r="B17" s="1">
+        <f t="shared" si="0"/>
+        <v>15</v>
+      </c>
+      <c r="C17" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="D17">
         <v>0.378</v>
       </c>
-      <c r="D17">
+      <c r="E17">
         <v>0.59646600000000005</v>
       </c>
     </row>
-    <row r="18" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A18" s="1">
         <v>16</v>
       </c>
-      <c r="B18" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="C18">
+      <c r="B18" s="1">
+        <f t="shared" si="0"/>
+        <v>16</v>
+      </c>
+      <c r="C18" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="D18">
         <v>0.376</v>
       </c>
-      <c r="D18">
+      <c r="E18">
         <v>0.71166099999999999</v>
       </c>
     </row>
-    <row r="19" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A19" s="1">
         <v>17</v>
       </c>
-      <c r="B19" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="C19">
+      <c r="B19" s="1">
+        <f t="shared" si="0"/>
+        <v>17</v>
+      </c>
+      <c r="C19" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="D19">
         <v>0.45650000000000002</v>
       </c>
-      <c r="D19">
+      <c r="E19">
         <v>0.74699599999999999</v>
       </c>
     </row>
-    <row r="20" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A20" s="1">
         <v>18</v>
       </c>
-      <c r="B20" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="C20">
+      <c r="B20" s="1">
+        <f t="shared" si="0"/>
+        <v>18</v>
+      </c>
+      <c r="C20" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="D20">
         <v>0.51249999999999996</v>
       </c>
-      <c r="D20">
+      <c r="E20">
         <v>0.74841000000000002</v>
       </c>
     </row>
-    <row r="21" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A21" s="1">
         <v>19</v>
       </c>
-      <c r="B21" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="C21">
+      <c r="B21" s="1">
+        <f t="shared" si="0"/>
+        <v>19</v>
+      </c>
+      <c r="C21" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="D21">
         <v>0.57999999999999996</v>
       </c>
-      <c r="D21">
+      <c r="E21">
         <v>0.491873</v>
       </c>
     </row>
-    <row r="22" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A22" s="1">
         <v>20</v>
       </c>
-      <c r="B22" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="C22">
+      <c r="B22" s="1">
+        <f t="shared" si="0"/>
+        <v>20</v>
+      </c>
+      <c r="C22" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="D22">
         <v>0.66949999999999998</v>
       </c>
-      <c r="D22">
+      <c r="E22">
         <v>0.491873</v>
       </c>
     </row>
-    <row r="23" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A23" s="1">
         <v>21</v>
       </c>
-      <c r="B23" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="C23">
+      <c r="B23" s="1">
+        <f t="shared" si="0"/>
+        <v>21</v>
+      </c>
+      <c r="C23" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="D23">
         <v>0.72650000000000003</v>
       </c>
-      <c r="D23">
+      <c r="E23">
         <v>0.49116599999999999</v>
       </c>
     </row>
-    <row r="24" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A24" s="1">
         <v>22</v>
       </c>
-      <c r="B24" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="C24">
+      <c r="B24" s="1">
+        <f t="shared" si="0"/>
+        <v>22</v>
+      </c>
+      <c r="C24" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="D24">
         <v>0.32750000000000001</v>
       </c>
-      <c r="D24">
+      <c r="E24">
         <v>0.35830400000000001</v>
       </c>
     </row>
-    <row r="25" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A25" s="1">
         <v>23</v>
       </c>
-      <c r="B25" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="C25">
+      <c r="B25" s="1">
+        <f t="shared" si="0"/>
+        <v>23</v>
+      </c>
+      <c r="C25" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="D25">
         <v>0.1895</v>
       </c>
-      <c r="D25">
+      <c r="E25">
         <v>0.39646599999999999</v>
       </c>
     </row>
-    <row r="26" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A26" s="1">
         <v>24</v>
       </c>
-      <c r="B26" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="C26">
+      <c r="B26" s="1">
+        <f t="shared" si="0"/>
+        <v>24</v>
+      </c>
+      <c r="C26" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="D26">
         <v>0.17199999999999999</v>
       </c>
-      <c r="D26">
+      <c r="E26">
         <v>0.68621900000000002</v>
       </c>
     </row>
-    <row r="27" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A27" s="1">
         <v>1120</v>
       </c>
-      <c r="B27" s="1" t="s">
-        <v>12</v>
-      </c>
-      <c r="C27">
+      <c r="B27" t="s">
+        <v>14</v>
+      </c>
+      <c r="C27" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="D27">
         <v>0.41099999999999998</v>
       </c>
-      <c r="D27">
+      <c r="E27">
         <v>0.41766799999999998</v>
       </c>
     </row>
-    <row r="28" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A28" s="1">
         <v>1160</v>
       </c>
-      <c r="B28" s="1" t="s">
-        <v>12</v>
-      </c>
-      <c r="C28">
+      <c r="B28" t="s">
+        <v>15</v>
+      </c>
+      <c r="C28" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="D28">
         <v>0.4375</v>
       </c>
-      <c r="D28">
+      <c r="E28">
         <v>0.87985899999999995</v>
       </c>
     </row>
-    <row r="29" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A29" s="1">
         <v>1160.01</v>
       </c>
-      <c r="B29" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="C29">
+      <c r="B29" s="1">
+        <f>A29</f>
+        <v>1160.01</v>
+      </c>
+      <c r="C29" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="D29">
         <v>0.39950000000000002</v>
       </c>
-      <c r="D29">
+      <c r="E29">
         <v>0.88127200000000006</v>
       </c>
     </row>
-    <row r="30" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A30" s="1">
         <v>1170</v>
       </c>
-      <c r="B30" s="1" t="s">
-        <v>12</v>
-      </c>
-      <c r="C30">
+      <c r="B30" t="s">
+        <v>16</v>
+      </c>
+      <c r="C30" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="D30">
         <v>0.439</v>
       </c>
-      <c r="D30">
+      <c r="E30">
         <v>0.951237</v>
       </c>
     </row>
-    <row r="31" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A31" s="1">
         <v>1180.01</v>
       </c>
-      <c r="B31" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="C31">
+      <c r="B31" s="1">
+        <f>A31</f>
+        <v>1180.01</v>
+      </c>
+      <c r="C31" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="D31">
         <v>8.9499999999999996E-2</v>
       </c>
-      <c r="D31">
+      <c r="E31">
         <v>0.16819799999999999</v>
       </c>
     </row>
-    <row r="32" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A32" s="1">
         <v>1180.02</v>
       </c>
-      <c r="B32" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="C32">
+      <c r="B32" s="1">
+        <f>A32</f>
+        <v>1180.02</v>
+      </c>
+      <c r="C32" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="D32">
         <v>9.0499999999999997E-2</v>
       </c>
-      <c r="D32">
+      <c r="E32">
         <v>0.187279</v>
       </c>
     </row>
-    <row r="33" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="33" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A33" s="1">
         <v>1180.03</v>
       </c>
-      <c r="B33" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="C33">
+      <c r="B33" s="1">
+        <f>A33</f>
+        <v>1180.03</v>
+      </c>
+      <c r="C33" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="D33">
         <v>8.8999999999999996E-2</v>
       </c>
-      <c r="D33">
+      <c r="E33">
         <v>0.208481</v>
       </c>
     </row>
-    <row r="34" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="34" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A34" s="1">
         <v>1181</v>
       </c>
-      <c r="B34" s="1" t="s">
-        <v>12</v>
-      </c>
-      <c r="C34">
+      <c r="B34" t="s">
+        <v>17</v>
+      </c>
+      <c r="C34" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="D34">
         <v>0.122</v>
       </c>
-      <c r="D34">
+      <c r="E34">
         <v>0.16819799999999999</v>
       </c>
     </row>
-    <row r="35" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="35" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A35" s="1">
         <v>1182</v>
       </c>
-      <c r="B35" s="1" t="s">
-        <v>12</v>
-      </c>
-      <c r="C35">
+      <c r="B35" t="s">
+        <v>18</v>
+      </c>
+      <c r="C35" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="D35">
         <v>0.122</v>
       </c>
-      <c r="D35">
+      <c r="E35">
         <v>0.18939900000000001</v>
       </c>
     </row>
-    <row r="36" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="36" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A36" s="1">
         <v>1191</v>
       </c>
-      <c r="B36" s="1" t="s">
-        <v>12</v>
-      </c>
-      <c r="C36">
+      <c r="B36" t="s">
+        <v>19</v>
+      </c>
+      <c r="C36" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="D36">
         <v>0.1225</v>
       </c>
-      <c r="D36">
+      <c r="E36">
         <v>0.20918700000000001</v>
       </c>
     </row>
-    <row r="37" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="37" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A37" s="1">
         <v>1192</v>
       </c>
-      <c r="B37" s="1" t="s">
-        <v>12</v>
-      </c>
-      <c r="C37">
+      <c r="B37" t="s">
+        <v>20</v>
+      </c>
+      <c r="C37" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="D37">
         <v>0.124</v>
       </c>
-      <c r="D37">
+      <c r="E37">
         <v>0.23038900000000001</v>
       </c>
     </row>
-    <row r="38" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="38" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A38" s="1">
         <v>3100.01</v>
       </c>
-      <c r="B38" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="C38">
+      <c r="B38" s="1">
+        <f>A38</f>
+        <v>3100.01</v>
+      </c>
+      <c r="C38" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="D38">
         <v>0.59699999999999998</v>
       </c>
-      <c r="D38">
+      <c r="E38">
         <v>0.18374599999999999</v>
       </c>
     </row>
-    <row r="39" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="39" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A39" s="1">
         <v>3100.02</v>
       </c>
-      <c r="B39" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="C39">
+      <c r="B39" s="1">
+        <f t="shared" ref="B39:B40" si="1">A39</f>
+        <v>3100.02</v>
+      </c>
+      <c r="C39" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="D39">
         <v>0.61450000000000005</v>
       </c>
-      <c r="D39">
+      <c r="E39">
         <v>0.25512400000000002</v>
       </c>
     </row>
-    <row r="40" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="40" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A40" s="1">
         <v>3100.03</v>
       </c>
-      <c r="B40" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="C40">
+      <c r="B40" s="1">
+        <f t="shared" si="1"/>
+        <v>3100.03</v>
+      </c>
+      <c r="C40" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="D40">
         <v>0.59550000000000003</v>
       </c>
-      <c r="D40">
+      <c r="E40">
         <v>0.23674899999999999</v>
       </c>
     </row>
-    <row r="41" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="41" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A41" s="1">
         <v>3101</v>
       </c>
-      <c r="B41" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="C41">
+      <c r="B41" t="s">
+        <v>21</v>
+      </c>
+      <c r="C41" s="1" t="s">
+        <v>55</v>
+      </c>
+      <c r="D41">
         <v>0.57550000000000001</v>
       </c>
-      <c r="D41">
+      <c r="E41">
         <v>0.236042</v>
       </c>
     </row>
-    <row r="42" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="42" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A42" s="1">
         <v>3102</v>
       </c>
-      <c r="B42" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="C42">
+      <c r="B42" t="s">
+        <v>22</v>
+      </c>
+      <c r="C42" s="1" t="s">
+        <v>55</v>
+      </c>
+      <c r="D42">
         <v>0.57399999999999995</v>
       </c>
-      <c r="D42">
+      <c r="E42">
         <v>0.30954100000000001</v>
       </c>
     </row>
-    <row r="43" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="43" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A43" s="1">
         <v>3150</v>
       </c>
-      <c r="B43" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="C43">
+      <c r="B43" t="s">
+        <v>23</v>
+      </c>
+      <c r="C43" s="1" t="s">
+        <v>55</v>
+      </c>
+      <c r="D43">
         <v>0.64749999999999996</v>
       </c>
-      <c r="D43">
+      <c r="E43">
         <v>0.26996500000000001</v>
       </c>
     </row>
-    <row r="44" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="44" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A44" s="1" t="s">
-        <v>11</v>
-      </c>
-      <c r="B44" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="C44">
+        <v>10</v>
+      </c>
+      <c r="B44" s="1" t="str">
+        <f>A44</f>
+        <v>3700.01</v>
+      </c>
+      <c r="C44" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="D44">
         <v>0.41099999999999998</v>
       </c>
-      <c r="D44">
+      <c r="E44">
         <v>0.39500000000000002</v>
       </c>
     </row>
-    <row r="45" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="45" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A45" s="1">
         <v>3800.01</v>
       </c>
-      <c r="B45" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="C45">
+      <c r="B45" s="1">
+        <f>A45</f>
+        <v>3800.01</v>
+      </c>
+      <c r="C45" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="D45">
         <v>0.58050000000000002</v>
       </c>
-      <c r="D45">
+      <c r="E45">
         <v>0.54911699999999997</v>
       </c>
     </row>
-    <row r="46" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="46" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A46" s="1">
         <v>3801</v>
       </c>
-      <c r="B46" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="C46">
+      <c r="B46" t="s">
+        <v>24</v>
+      </c>
+      <c r="C46" s="1" t="s">
+        <v>55</v>
+      </c>
+      <c r="D46">
         <v>0.54749999999999999</v>
       </c>
-      <c r="D46">
+      <c r="E46">
         <v>0.56113100000000005</v>
       </c>
     </row>
-    <row r="47" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="47" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A47" s="1">
         <v>3806</v>
       </c>
-      <c r="B47" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="C47">
+      <c r="B47" t="s">
+        <v>25</v>
+      </c>
+      <c r="C47" s="1" t="s">
+        <v>55</v>
+      </c>
+      <c r="D47">
         <v>0.61250000000000004</v>
       </c>
-      <c r="D47">
+      <c r="E47">
         <v>0.54629000000000005</v>
       </c>
     </row>
-    <row r="48" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="48" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A48" s="1">
         <v>3900.01</v>
       </c>
-      <c r="B48" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="C48">
+      <c r="B48" s="1">
+        <f>A48</f>
+        <v>3900.01</v>
+      </c>
+      <c r="C48" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="D48">
         <v>0.505</v>
       </c>
-      <c r="D48">
+      <c r="E48">
         <v>0.53639599999999998</v>
       </c>
     </row>
-    <row r="49" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="49" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A49" s="1">
         <v>3900.02</v>
       </c>
-      <c r="B49" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="C49">
+      <c r="B49" s="1">
+        <f t="shared" ref="B49:B50" si="2">A49</f>
+        <v>3900.02</v>
+      </c>
+      <c r="C49" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="D49">
         <v>0.50600000000000001</v>
       </c>
-      <c r="D49">
+      <c r="E49">
         <v>0.58374599999999999</v>
       </c>
     </row>
-    <row r="50" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="50" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A50" s="1">
         <v>3900.03</v>
       </c>
-      <c r="B50" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="C50">
+      <c r="B50" s="1">
+        <f t="shared" si="2"/>
+        <v>3900.03</v>
+      </c>
+      <c r="C50" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="D50">
         <v>0.50949999999999995</v>
       </c>
-      <c r="D50">
+      <c r="E50">
         <v>0.67137800000000003</v>
       </c>
     </row>
-    <row r="51" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="51" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A51" s="1">
         <v>3901</v>
       </c>
-      <c r="B51" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="C51">
+      <c r="B51" t="s">
+        <v>26</v>
+      </c>
+      <c r="C51" s="1" t="s">
+        <v>55</v>
+      </c>
+      <c r="D51">
         <v>0.52149999999999996</v>
       </c>
-      <c r="D51">
+      <c r="E51">
         <v>0.58374599999999999</v>
       </c>
     </row>
-    <row r="52" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="52" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A52" s="1">
         <v>3906</v>
       </c>
-      <c r="B52" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="C52">
+      <c r="B52" t="s">
+        <v>27</v>
+      </c>
+      <c r="C52" s="1" t="s">
+        <v>55</v>
+      </c>
+      <c r="D52">
         <v>0.49149999999999999</v>
       </c>
-      <c r="D52">
+      <c r="E52">
         <v>0.700353</v>
       </c>
     </row>
-    <row r="53" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="53" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A53" s="1">
         <v>4200.01</v>
       </c>
-      <c r="B53" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="C53">
+      <c r="B53" s="1">
+        <f>A53</f>
+        <v>4200.01</v>
+      </c>
+      <c r="C53" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="D53">
         <v>0.67</v>
       </c>
-      <c r="D53">
+      <c r="E53">
         <v>0.53568899999999997</v>
       </c>
     </row>
-    <row r="54" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="54" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A54" s="1">
         <v>4201</v>
       </c>
-      <c r="B54" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="C54">
+      <c r="B54" t="s">
+        <v>52</v>
+      </c>
+      <c r="C54" s="1" t="s">
+        <v>55</v>
+      </c>
+      <c r="D54">
         <v>0.66900000000000004</v>
       </c>
-      <c r="D54">
+      <c r="E54">
         <v>0.57950500000000005</v>
       </c>
     </row>
-    <row r="55" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="55" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A55" s="1">
         <v>4202</v>
       </c>
-      <c r="B55" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="C55">
+      <c r="B55" t="s">
+        <v>53</v>
+      </c>
+      <c r="C55" s="1" t="s">
+        <v>55</v>
+      </c>
+      <c r="D55">
         <v>0.66449999999999998</v>
       </c>
-      <c r="D55">
+      <c r="E55">
         <v>0.55476999999999999</v>
       </c>
     </row>
-    <row r="56" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="56" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A56" s="1">
         <v>4300.01</v>
       </c>
-      <c r="B56" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="C56">
+      <c r="B56" s="1">
+        <f>A56</f>
+        <v>4300.01</v>
+      </c>
+      <c r="C56" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="D56">
         <v>0.72750000000000004</v>
       </c>
-      <c r="D56">
+      <c r="E56">
         <v>0.52932900000000005</v>
       </c>
     </row>
-    <row r="57" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="57" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A57" s="1">
         <v>4303</v>
       </c>
-      <c r="B57" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="C57">
+      <c r="B57" t="s">
+        <v>28</v>
+      </c>
+      <c r="C57" s="1" t="s">
+        <v>55</v>
+      </c>
+      <c r="D57">
         <v>0.71699999999999997</v>
       </c>
-      <c r="D57">
+      <c r="E57">
         <v>0.56537099999999996</v>
       </c>
     </row>
-    <row r="58" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="58" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A58" s="1">
         <v>4304</v>
       </c>
-      <c r="B58" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="C58">
+      <c r="B58" t="s">
+        <v>29</v>
+      </c>
+      <c r="C58" s="1" t="s">
+        <v>55</v>
+      </c>
+      <c r="D58">
         <v>0.71599999999999997</v>
       </c>
-      <c r="D58">
+      <c r="E58">
         <v>0.53003500000000003</v>
       </c>
     </row>
-    <row r="59" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="59" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A59" s="1">
         <v>4501</v>
       </c>
-      <c r="B59" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="C59">
+      <c r="B59" t="s">
+        <v>30</v>
+      </c>
+      <c r="C59" s="1" t="s">
+        <v>55</v>
+      </c>
+      <c r="D59">
         <v>0.4365</v>
       </c>
-      <c r="D59">
+      <c r="E59">
         <v>0.66219099999999997</v>
       </c>
     </row>
-    <row r="60" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A60" s="1">
+    <row r="60" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A60" s="1" t="s">
+        <v>56</v>
+      </c>
+      <c r="B60" s="1" t="str">
+        <f>A60</f>
+        <v>4600.02</v>
+      </c>
+      <c r="C60" s="1" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="61" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A61" s="1">
         <v>4651</v>
       </c>
-      <c r="B60" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="C60">
+      <c r="B61" t="s">
+        <v>31</v>
+      </c>
+      <c r="C61" s="1" t="s">
+        <v>55</v>
+      </c>
+      <c r="D61">
         <v>0.35199999999999998</v>
       </c>
-      <c r="D60">
+      <c r="E61">
         <v>0.75123700000000004</v>
       </c>
     </row>
-    <row r="61" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A61" s="1">
+    <row r="62" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A62" s="1" t="s">
+        <v>57</v>
+      </c>
+      <c r="B62" s="1" t="str">
+        <f>A62</f>
+        <v>4600.01</v>
+      </c>
+      <c r="C62" s="1" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="63" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A63" s="1">
         <v>4671</v>
       </c>
-      <c r="B61" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="C61">
+      <c r="B63" t="s">
+        <v>32</v>
+      </c>
+      <c r="C63" s="1" t="s">
+        <v>55</v>
+      </c>
+      <c r="D63">
         <v>0.34949999999999998</v>
       </c>
-      <c r="D61">
+      <c r="E63">
         <v>0.68763300000000005</v>
       </c>
     </row>
-    <row r="62" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A62" s="1">
+    <row r="64" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A64" s="1">
         <v>4700.01</v>
       </c>
-      <c r="B62" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="C62">
+      <c r="B64" s="1">
+        <f>A64</f>
+        <v>4700.01</v>
+      </c>
+      <c r="C64" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="D64">
         <v>0.41449999999999998</v>
       </c>
-      <c r="D62">
+      <c r="E64">
         <v>0.56961099999999998</v>
       </c>
     </row>
-    <row r="63" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A63" s="1">
+    <row r="65" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A65" s="1">
         <v>4700.0200000000004</v>
       </c>
-      <c r="B63" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="C63">
+      <c r="B65" s="1">
+        <f>A65</f>
+        <v>4700.0200000000004</v>
+      </c>
+      <c r="C65" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="D65">
         <v>0.42849999999999999</v>
       </c>
-      <c r="D63">
+      <c r="E65">
         <v>0.57314500000000002</v>
       </c>
     </row>
-    <row r="64" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A64" s="1">
+    <row r="66" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A66" s="1">
         <v>4710</v>
       </c>
-      <c r="B64" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="C64">
+      <c r="B66" t="s">
+        <v>33</v>
+      </c>
+      <c r="C66" s="1" t="s">
+        <v>55</v>
+      </c>
+      <c r="D66">
         <v>0.44750000000000001</v>
       </c>
-      <c r="D64">
+      <c r="E66">
         <v>0.57526500000000003</v>
       </c>
     </row>
-    <row r="65" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A65" s="1">
+    <row r="67" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A67" s="1">
         <v>4740</v>
       </c>
-      <c r="B65" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="C65">
+      <c r="B67" t="s">
+        <v>34</v>
+      </c>
+      <c r="C67" s="1" t="s">
+        <v>55</v>
+      </c>
+      <c r="D67">
         <v>0.45150000000000001</v>
       </c>
-      <c r="D65">
+      <c r="E67">
         <v>0.61342799999999997</v>
       </c>
     </row>
-    <row r="66" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A66" s="1">
+    <row r="68" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A68" s="1">
         <v>4810</v>
       </c>
-      <c r="B66" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="C66">
+      <c r="B68" t="s">
+        <v>35</v>
+      </c>
+      <c r="C68" s="1" t="s">
+        <v>55</v>
+      </c>
+      <c r="D68">
         <v>0.44350000000000001</v>
       </c>
-      <c r="D66">
+      <c r="E68">
         <v>0.542049</v>
       </c>
     </row>
-    <row r="67" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A67" s="1">
+    <row r="69" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A69" s="1">
         <v>5600</v>
       </c>
-      <c r="B67" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="C67">
+      <c r="B69" t="s">
+        <v>36</v>
+      </c>
+      <c r="C69" s="1" t="s">
+        <v>55</v>
+      </c>
+      <c r="D69">
         <v>0.154</v>
       </c>
-      <c r="D67">
+      <c r="E69">
         <v>0.39293299999999998</v>
       </c>
     </row>
-    <row r="68" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A68" s="1">
+    <row r="70" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A70" s="1">
         <v>5700.01</v>
       </c>
-      <c r="B68" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="C68">
+      <c r="B70" s="1">
+        <f>A70</f>
+        <v>5700.01</v>
+      </c>
+      <c r="C70" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="D70">
         <v>0.51300000000000001</v>
       </c>
-      <c r="D68">
+      <c r="E70">
         <v>0.403534</v>
       </c>
     </row>
-    <row r="69" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A69" s="1">
+    <row r="71" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A71" s="1">
         <v>5701</v>
       </c>
-      <c r="B69" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="C69">
+      <c r="B71" t="s">
+        <v>37</v>
+      </c>
+      <c r="C71" s="1" t="s">
+        <v>55</v>
+      </c>
+      <c r="D71">
         <v>0.47</v>
       </c>
-      <c r="D69">
+      <c r="E71">
         <v>0.41625400000000001</v>
       </c>
     </row>
-    <row r="70" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A70" s="1">
+    <row r="72" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A72" s="1">
         <v>5800.01</v>
       </c>
-      <c r="B70" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="C70">
+      <c r="B72" s="1">
+        <f>A72</f>
+        <v>5800.01</v>
+      </c>
+      <c r="C72" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="D72">
         <v>0.39600000000000002</v>
       </c>
-      <c r="D70">
+      <c r="E72">
         <v>0.48056500000000002</v>
       </c>
     </row>
-    <row r="71" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A71" s="1">
+    <row r="73" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A73" s="1">
         <v>5801</v>
       </c>
-      <c r="B71" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="C71">
+      <c r="B73" t="s">
+        <v>38</v>
+      </c>
+      <c r="C73" s="1" t="s">
+        <v>55</v>
+      </c>
+      <c r="D73">
         <v>0.37</v>
       </c>
-      <c r="D71">
+      <c r="E73">
         <v>0.482686</v>
       </c>
     </row>
-    <row r="72" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A72" s="1">
+    <row r="74" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A74" s="1">
         <v>5802</v>
       </c>
-      <c r="B72" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="C72">
+      <c r="B74" t="s">
+        <v>39</v>
+      </c>
+      <c r="C74" s="1" t="s">
+        <v>55</v>
+      </c>
+      <c r="D74">
         <v>0.37</v>
       </c>
-      <c r="D72">
+      <c r="E74">
         <v>0.46219100000000002</v>
       </c>
     </row>
-    <row r="73" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A73" s="1">
+    <row r="75" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A75" s="1">
         <v>8104</v>
       </c>
-      <c r="B73" s="1" t="s">
+      <c r="B75" t="s">
+        <v>40</v>
+      </c>
+      <c r="C75" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="C73">
+      <c r="D75">
         <v>0.3095</v>
       </c>
-      <c r="D73">
+      <c r="E75">
         <v>2.4735E-2</v>
       </c>
     </row>
-    <row r="74" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A74" s="1">
+    <row r="76" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A76" s="1">
         <v>8105</v>
       </c>
-      <c r="B74" s="1" t="s">
+      <c r="B76" t="s">
+        <v>41</v>
+      </c>
+      <c r="C76" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="C74">
+      <c r="D76">
         <v>0.16450000000000001</v>
       </c>
-      <c r="D74">
+      <c r="E76">
         <v>2.1201000000000001E-2</v>
       </c>
     </row>
-    <row r="75" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A75" s="1">
+    <row r="77" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A77" s="1">
         <v>8106</v>
       </c>
-      <c r="B75" s="1" t="s">
+      <c r="B77" t="s">
+        <v>42</v>
+      </c>
+      <c r="C77" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="C75">
+      <c r="D77">
         <v>0.3105</v>
       </c>
-      <c r="D75">
+      <c r="E77">
         <v>7.4204999999999993E-2</v>
       </c>
     </row>
-    <row r="76" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A76" s="1">
+    <row r="78" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A78" s="1">
         <v>8107</v>
       </c>
-      <c r="B76" s="1" t="s">
+      <c r="B78" t="s">
+        <v>43</v>
+      </c>
+      <c r="C78" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="C76">
+      <c r="D78">
         <v>0.16350000000000001</v>
       </c>
-      <c r="D76">
+      <c r="E78">
         <v>6.9964999999999999E-2</v>
       </c>
     </row>
-    <row r="77" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A77" s="1">
+    <row r="79" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A79" s="1">
         <v>8108</v>
       </c>
-      <c r="B77" s="1" t="s">
+      <c r="B79" t="s">
+        <v>44</v>
+      </c>
+      <c r="C79" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="C77">
+      <c r="D79">
         <v>0.3095</v>
       </c>
-      <c r="D77">
+      <c r="E79">
         <v>4.3816000000000001E-2</v>
       </c>
     </row>
-    <row r="78" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A78" s="1">
+    <row r="80" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A80" s="1">
         <v>8109</v>
       </c>
-      <c r="B78" s="1" t="s">
+      <c r="B80" t="s">
+        <v>45</v>
+      </c>
+      <c r="C80" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="C78">
+      <c r="D80">
         <v>0.39950000000000002</v>
       </c>
-      <c r="D78">
+      <c r="E80">
         <v>0.79788000000000003</v>
       </c>
     </row>
-    <row r="79" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A79" s="1">
+    <row r="81" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A81" s="1">
         <v>31001</v>
       </c>
-      <c r="B79" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="C79">
+      <c r="B81" t="s">
+        <v>46</v>
+      </c>
+      <c r="C81" s="1" t="s">
+        <v>55</v>
+      </c>
+      <c r="D81">
         <v>0.52149999999999996</v>
       </c>
-      <c r="D79">
+      <c r="E81">
         <v>0.53639599999999998</v>
       </c>
     </row>
-    <row r="80" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A80" s="1">
+    <row r="82" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A82" s="1">
         <v>31006</v>
       </c>
-      <c r="B80" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="C80">
+      <c r="B82" t="s">
+        <v>47</v>
+      </c>
+      <c r="C82" s="1" t="s">
+        <v>55</v>
+      </c>
+      <c r="D82">
         <v>0.48749999999999999</v>
       </c>
-      <c r="D80">
+      <c r="E82">
         <v>0.67349800000000004</v>
       </c>
     </row>
-    <row r="81" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A81" s="1">
+    <row r="83" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A83" s="1">
         <v>51000</v>
       </c>
-      <c r="B81" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="C81">
+      <c r="B83" t="s">
+        <v>48</v>
+      </c>
+      <c r="C83" s="1" t="s">
+        <v>55</v>
+      </c>
+      <c r="D83">
         <v>0.28399999999999997</v>
       </c>
-      <c r="D81">
+      <c r="E83">
         <v>0.187279</v>
       </c>
     </row>
-    <row r="82" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A82" s="1">
+    <row r="84" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A84" s="1">
         <v>52100.01</v>
       </c>
-      <c r="B82" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="C82">
+      <c r="B84" s="1">
+        <f>A84</f>
+        <v>52100.01</v>
+      </c>
+      <c r="C84" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="D84">
         <v>0.14149999999999999</v>
       </c>
-      <c r="D82">
+      <c r="E84">
         <v>0.67491199999999996</v>
       </c>
     </row>
-    <row r="83" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A83" s="1">
+    <row r="85" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A85" s="1">
         <v>52100.02</v>
       </c>
-      <c r="B83" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="C83">
+      <c r="B85" s="1">
+        <f>A85</f>
+        <v>52100.02</v>
+      </c>
+      <c r="C85" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="D85">
         <v>0.1195</v>
       </c>
-      <c r="D83">
+      <c r="E85">
         <v>0.67137800000000003</v>
       </c>
     </row>
-    <row r="84" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A84" s="1">
+    <row r="86" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A86" s="1">
         <v>52107</v>
       </c>
-      <c r="B84" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="C84">
+      <c r="B86" t="s">
+        <v>50</v>
+      </c>
+      <c r="C86" s="1" t="s">
+        <v>55</v>
+      </c>
+      <c r="D86">
         <v>0.104</v>
       </c>
-      <c r="D84">
+      <c r="E86">
         <v>0.62897499999999995</v>
       </c>
     </row>
-    <row r="85" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A85" s="1">
+    <row r="87" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A87" s="1">
         <v>52207</v>
       </c>
-      <c r="B85" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="C85">
+      <c r="B87" t="s">
+        <v>51</v>
+      </c>
+      <c r="C87" s="1" t="s">
+        <v>55</v>
+      </c>
+      <c r="D87">
         <v>0.1195</v>
       </c>
-      <c r="D85">
+      <c r="E87">
         <v>0.63250899999999999</v>
       </c>
     </row>
-    <row r="86" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A86" s="1">
+    <row r="88" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A88" s="1">
         <v>53000</v>
       </c>
-      <c r="B86" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="C86">
+      <c r="B88" t="s">
+        <v>49</v>
+      </c>
+      <c r="C88" s="1" t="s">
+        <v>55</v>
+      </c>
+      <c r="D88">
         <v>0.25600000000000001</v>
       </c>
-      <c r="D86">
+      <c r="E88">
         <v>0.17879900000000001</v>
       </c>
     </row>
-    <row r="87" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A87" s="1">
+    <row r="89" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A89" s="1">
         <v>56000</v>
       </c>
-      <c r="B87" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="C87">
+      <c r="B89" t="s">
+        <v>54</v>
+      </c>
+      <c r="C89" s="1" t="s">
+        <v>55</v>
+      </c>
+      <c r="D89">
         <v>0.11799999999999999</v>
       </c>
-      <c r="D87">
+      <c r="E89">
         <v>0.76749100000000003</v>
       </c>
     </row>
   </sheetData>
+  <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="8" orientation="landscape" r:id="rId1"/>
 </worksheet>
 </file>
 
@@ -2714,7 +3187,7 @@
         <v>1182</v>
       </c>
       <c r="C86" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
     </row>
     <row r="87" spans="1:3" x14ac:dyDescent="0.3">
@@ -2726,7 +3199,7 @@
         <v>1191</v>
       </c>
       <c r="C87" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
     </row>
     <row r="88" spans="1:3" x14ac:dyDescent="0.3">
@@ -2738,7 +3211,7 @@
         <v>1192</v>
       </c>
       <c r="C88" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
     </row>
     <row r="89" spans="1:3" x14ac:dyDescent="0.3">
@@ -2750,7 +3223,7 @@
         <v>3100.01</v>
       </c>
       <c r="C89" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
     </row>
     <row r="90" spans="1:3" x14ac:dyDescent="0.3">
@@ -2762,7 +3235,7 @@
         <v/>
       </c>
       <c r="C90" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
     </row>
     <row r="91" spans="1:3" x14ac:dyDescent="0.3">
@@ -2774,7 +3247,7 @@
         <v/>
       </c>
       <c r="C91" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
     </row>
     <row r="92" spans="1:3" x14ac:dyDescent="0.3">
@@ -2786,7 +3259,7 @@
         <v>3100.02</v>
       </c>
       <c r="C92" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
     </row>
     <row r="93" spans="1:3" x14ac:dyDescent="0.3">
@@ -2798,7 +3271,7 @@
         <v/>
       </c>
       <c r="C93" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
     </row>
     <row r="94" spans="1:3" x14ac:dyDescent="0.3">
@@ -2810,7 +3283,7 @@
         <v>3100.03</v>
       </c>
       <c r="C94" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
     </row>
     <row r="95" spans="1:3" x14ac:dyDescent="0.3">
@@ -2822,7 +3295,7 @@
         <v/>
       </c>
       <c r="C95" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
     </row>
     <row r="96" spans="1:3" x14ac:dyDescent="0.3">
@@ -2834,7 +3307,7 @@
         <v/>
       </c>
       <c r="C96" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
     </row>
     <row r="97" spans="1:3" x14ac:dyDescent="0.3">
@@ -2846,7 +3319,7 @@
         <v>3101</v>
       </c>
       <c r="C97" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
     </row>
     <row r="98" spans="1:3" x14ac:dyDescent="0.3">
@@ -2858,7 +3331,7 @@
         <v>3102</v>
       </c>
       <c r="C98" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
     </row>
     <row r="99" spans="1:3" x14ac:dyDescent="0.3">
@@ -2870,7 +3343,7 @@
         <v>3150</v>
       </c>
       <c r="C99" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
     </row>
     <row r="100" spans="1:3" x14ac:dyDescent="0.3">
@@ -2882,7 +3355,7 @@
         <v>3800.01</v>
       </c>
       <c r="C100" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
     </row>
     <row r="101" spans="1:3" x14ac:dyDescent="0.3">
@@ -2894,7 +3367,7 @@
         <v/>
       </c>
       <c r="C101" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
     </row>
     <row r="102" spans="1:3" x14ac:dyDescent="0.3">
@@ -2906,7 +3379,7 @@
         <v/>
       </c>
       <c r="C102" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
     </row>
     <row r="103" spans="1:3" x14ac:dyDescent="0.3">
@@ -2918,7 +3391,7 @@
         <v>3801</v>
       </c>
       <c r="C103" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
     </row>
     <row r="104" spans="1:3" x14ac:dyDescent="0.3">
@@ -2930,7 +3403,7 @@
         <v>3806</v>
       </c>
       <c r="C104" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
     </row>
     <row r="105" spans="1:3" x14ac:dyDescent="0.3">
@@ -2942,7 +3415,7 @@
         <v>3900.01</v>
       </c>
       <c r="C105" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
     </row>
     <row r="106" spans="1:3" x14ac:dyDescent="0.3">
@@ -2954,7 +3427,7 @@
         <v/>
       </c>
       <c r="C106" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
     </row>
     <row r="107" spans="1:3" x14ac:dyDescent="0.3">
@@ -2966,7 +3439,7 @@
         <v/>
       </c>
       <c r="C107" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
     </row>
     <row r="108" spans="1:3" x14ac:dyDescent="0.3">
@@ -2978,7 +3451,7 @@
         <v>3900.02</v>
       </c>
       <c r="C108" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
     </row>
     <row r="109" spans="1:3" x14ac:dyDescent="0.3">
@@ -2990,7 +3463,7 @@
         <v/>
       </c>
       <c r="C109" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
     </row>
     <row r="110" spans="1:3" x14ac:dyDescent="0.3">
@@ -3002,7 +3475,7 @@
         <v/>
       </c>
       <c r="C110" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
     </row>
     <row r="111" spans="1:3" x14ac:dyDescent="0.3">
@@ -3014,7 +3487,7 @@
         <v>3900.03</v>
       </c>
       <c r="C111" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
     </row>
     <row r="112" spans="1:3" x14ac:dyDescent="0.3">
@@ -3026,7 +3499,7 @@
         <v/>
       </c>
       <c r="C112" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
     </row>
     <row r="113" spans="1:3" x14ac:dyDescent="0.3">
@@ -3038,7 +3511,7 @@
         <v/>
       </c>
       <c r="C113" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
     </row>
     <row r="114" spans="1:3" x14ac:dyDescent="0.3">
@@ -3050,7 +3523,7 @@
         <v>3901</v>
       </c>
       <c r="C114" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
     </row>
     <row r="115" spans="1:3" x14ac:dyDescent="0.3">
@@ -3062,7 +3535,7 @@
         <v>3906</v>
       </c>
       <c r="C115" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
     </row>
     <row r="116" spans="1:3" x14ac:dyDescent="0.3">
@@ -3074,7 +3547,7 @@
         <v>4200.01</v>
       </c>
       <c r="C116" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
     </row>
     <row r="117" spans="1:3" x14ac:dyDescent="0.3">
@@ -3086,7 +3559,7 @@
         <v/>
       </c>
       <c r="C117" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
     </row>
     <row r="118" spans="1:3" x14ac:dyDescent="0.3">
@@ -3098,7 +3571,7 @@
         <v/>
       </c>
       <c r="C118" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
     </row>
     <row r="119" spans="1:3" x14ac:dyDescent="0.3">
@@ -3110,7 +3583,7 @@
         <v>4201</v>
       </c>
       <c r="C119" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
     </row>
     <row r="120" spans="1:3" x14ac:dyDescent="0.3">
@@ -3122,7 +3595,7 @@
         <v>4202</v>
       </c>
       <c r="C120" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
     </row>
     <row r="121" spans="1:3" x14ac:dyDescent="0.3">
@@ -3134,7 +3607,7 @@
         <v>4300.01</v>
       </c>
       <c r="C121" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
     </row>
     <row r="122" spans="1:3" x14ac:dyDescent="0.3">
@@ -3146,7 +3619,7 @@
         <v/>
       </c>
       <c r="C122" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
     </row>
     <row r="123" spans="1:3" x14ac:dyDescent="0.3">
@@ -3158,7 +3631,7 @@
         <v/>
       </c>
       <c r="C123" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
     </row>
     <row r="124" spans="1:3" x14ac:dyDescent="0.3">
@@ -3170,7 +3643,7 @@
         <v>4303</v>
       </c>
       <c r="C124" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
     </row>
     <row r="125" spans="1:3" x14ac:dyDescent="0.3">
@@ -3182,7 +3655,7 @@
         <v>4304</v>
       </c>
       <c r="C125" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
     </row>
     <row r="126" spans="1:3" x14ac:dyDescent="0.3">
@@ -3194,7 +3667,7 @@
         <v>4501</v>
       </c>
       <c r="C126" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
     </row>
     <row r="127" spans="1:3" x14ac:dyDescent="0.3">
@@ -3206,7 +3679,7 @@
         <v>4651</v>
       </c>
       <c r="C127" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
     </row>
     <row r="128" spans="1:3" x14ac:dyDescent="0.3">
@@ -3218,7 +3691,7 @@
         <v>4671</v>
       </c>
       <c r="C128" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
     </row>
     <row r="129" spans="1:3" x14ac:dyDescent="0.3">
@@ -3230,7 +3703,7 @@
         <v>4700.01</v>
       </c>
       <c r="C129" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
     </row>
     <row r="130" spans="1:3" x14ac:dyDescent="0.3">
@@ -3242,7 +3715,7 @@
         <v/>
       </c>
       <c r="C130" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
     </row>
     <row r="131" spans="1:3" x14ac:dyDescent="0.3">
@@ -3254,7 +3727,7 @@
         <v/>
       </c>
       <c r="C131" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
     </row>
     <row r="132" spans="1:3" x14ac:dyDescent="0.3">
@@ -3266,7 +3739,7 @@
         <v>4700.0200000000004</v>
       </c>
       <c r="C132" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
     </row>
     <row r="133" spans="1:3" x14ac:dyDescent="0.3">
@@ -3278,7 +3751,7 @@
         <v/>
       </c>
       <c r="C133" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
     </row>
     <row r="134" spans="1:3" x14ac:dyDescent="0.3">
@@ -3290,7 +3763,7 @@
         <v/>
       </c>
       <c r="C134" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
     </row>
     <row r="135" spans="1:3" x14ac:dyDescent="0.3">
@@ -3302,7 +3775,7 @@
         <v>4710</v>
       </c>
       <c r="C135" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
     </row>
     <row r="136" spans="1:3" x14ac:dyDescent="0.3">
@@ -3314,7 +3787,7 @@
         <v>4740</v>
       </c>
       <c r="C136" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
     </row>
     <row r="137" spans="1:3" x14ac:dyDescent="0.3">
@@ -3326,7 +3799,7 @@
         <v>4810</v>
       </c>
       <c r="C137" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
     </row>
     <row r="138" spans="1:3" x14ac:dyDescent="0.3">
@@ -3338,7 +3811,7 @@
         <v>5600</v>
       </c>
       <c r="C138" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
     </row>
     <row r="139" spans="1:3" x14ac:dyDescent="0.3">
@@ -3350,7 +3823,7 @@
         <v>5700.01</v>
       </c>
       <c r="C139" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
     </row>
     <row r="140" spans="1:3" x14ac:dyDescent="0.3">
@@ -3362,7 +3835,7 @@
         <v/>
       </c>
       <c r="C140" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
     </row>
     <row r="141" spans="1:3" x14ac:dyDescent="0.3">
@@ -3374,7 +3847,7 @@
         <v>5701</v>
       </c>
       <c r="C141" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
     </row>
     <row r="142" spans="1:3" x14ac:dyDescent="0.3">
@@ -3386,7 +3859,7 @@
         <v>5800.01</v>
       </c>
       <c r="C142" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
     </row>
     <row r="143" spans="1:3" x14ac:dyDescent="0.3">
@@ -3398,7 +3871,7 @@
         <v/>
       </c>
       <c r="C143" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
     </row>
     <row r="144" spans="1:3" x14ac:dyDescent="0.3">
@@ -3410,7 +3883,7 @@
         <v/>
       </c>
       <c r="C144" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
     </row>
     <row r="145" spans="1:3" x14ac:dyDescent="0.3">
@@ -3422,7 +3895,7 @@
         <v>5801</v>
       </c>
       <c r="C145" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
     </row>
     <row r="146" spans="1:3" x14ac:dyDescent="0.3">
@@ -3434,7 +3907,7 @@
         <v>5802</v>
       </c>
       <c r="C146" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
     </row>
     <row r="147" spans="1:3" x14ac:dyDescent="0.3">
@@ -3446,7 +3919,7 @@
         <v>8104</v>
       </c>
       <c r="C147" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
     </row>
     <row r="148" spans="1:3" x14ac:dyDescent="0.3">
@@ -3458,7 +3931,7 @@
         <v>8105</v>
       </c>
       <c r="C148" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
     </row>
     <row r="149" spans="1:3" x14ac:dyDescent="0.3">
@@ -3470,7 +3943,7 @@
         <v>8106</v>
       </c>
       <c r="C149" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
     </row>
     <row r="150" spans="1:3" x14ac:dyDescent="0.3">
@@ -3482,7 +3955,7 @@
         <v>8107</v>
       </c>
       <c r="C150" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
     </row>
     <row r="151" spans="1:3" x14ac:dyDescent="0.3">
@@ -3494,7 +3967,7 @@
         <v>8108</v>
       </c>
       <c r="C151" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
     </row>
     <row r="152" spans="1:3" x14ac:dyDescent="0.3">
@@ -3506,7 +3979,7 @@
         <v>8109</v>
       </c>
       <c r="C152" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
     </row>
     <row r="153" spans="1:3" x14ac:dyDescent="0.3">
@@ -3518,7 +3991,7 @@
         <v>31001</v>
       </c>
       <c r="C153" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
     </row>
     <row r="154" spans="1:3" x14ac:dyDescent="0.3">
@@ -3530,7 +4003,7 @@
         <v>31006</v>
       </c>
       <c r="C154" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
     </row>
     <row r="155" spans="1:3" x14ac:dyDescent="0.3">
@@ -3542,7 +4015,7 @@
         <v>51000</v>
       </c>
       <c r="C155" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
     </row>
     <row r="156" spans="1:3" x14ac:dyDescent="0.3">
@@ -3554,7 +4027,7 @@
         <v>52100.01</v>
       </c>
       <c r="C156" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
     </row>
     <row r="157" spans="1:3" x14ac:dyDescent="0.3">
@@ -3566,7 +4039,7 @@
         <v/>
       </c>
       <c r="C157" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
     </row>
     <row r="158" spans="1:3" x14ac:dyDescent="0.3">
@@ -3578,7 +4051,7 @@
         <v>52100.02</v>
       </c>
       <c r="C158" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
     </row>
     <row r="159" spans="1:3" x14ac:dyDescent="0.3">
@@ -3590,7 +4063,7 @@
         <v/>
       </c>
       <c r="C159" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
     </row>
     <row r="160" spans="1:3" x14ac:dyDescent="0.3">
@@ -3602,7 +4075,7 @@
         <v/>
       </c>
       <c r="C160" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
     </row>
     <row r="161" spans="1:3" x14ac:dyDescent="0.3">
@@ -3614,7 +4087,7 @@
         <v>52107</v>
       </c>
       <c r="C161" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
     </row>
     <row r="162" spans="1:3" x14ac:dyDescent="0.3">
@@ -3626,7 +4099,7 @@
         <v>52207</v>
       </c>
       <c r="C162" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
     </row>
     <row r="163" spans="1:3" x14ac:dyDescent="0.3">
@@ -3638,7 +4111,7 @@
         <v>53000</v>
       </c>
       <c r="C163" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
     </row>
     <row r="164" spans="1:3" x14ac:dyDescent="0.3">

</xml_diff>